<commit_message>
performed new update for quick analysis on megamillions game
</commit_message>
<xml_diff>
--- a/mega_millions_draws.xlsx
+++ b/mega_millions_draws.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2509"/>
+  <dimension ref="A1:L2510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -101730,6 +101730,44 @@
       </c>
       <c r="L2509" t="inlineStr"/>
     </row>
+    <row r="2510">
+      <c r="A2510" s="2" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B2510" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C2510" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2510" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2510" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="F2510" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2510" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2510" t="n">
+        <v>36</v>
+      </c>
+      <c r="I2510" t="n">
+        <v>38</v>
+      </c>
+      <c r="J2510" t="n">
+        <v>40</v>
+      </c>
+      <c r="K2510" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2510" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Powerball data through 8/8/2026
Backfilled the missing 8/5 draw (14-20-59-60-61, PB 25) and appended
the 8/8 draw (05-09-35-54-63, PB 7) to powerball_game.xlsx, and
repointed the draw-audit example at the 8/8 result.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mega_millions_draws.xlsx
+++ b/mega_millions_draws.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2522"/>
+  <dimension ref="A1:L2525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -102212,6 +102212,120 @@
       </c>
       <c r="L2522" t="inlineStr"/>
     </row>
+    <row r="2523">
+      <c r="A2523" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B2523" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C2523" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2523" t="n">
+        <v>24</v>
+      </c>
+      <c r="E2523" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="F2523" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2523" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2523" t="n">
+        <v>42</v>
+      </c>
+      <c r="I2523" t="n">
+        <v>44</v>
+      </c>
+      <c r="J2523" t="n">
+        <v>60</v>
+      </c>
+      <c r="K2523" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2523" t="inlineStr"/>
+    </row>
+    <row r="2524">
+      <c r="A2524" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B2524" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C2524" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2524" t="n">
+        <v>28</v>
+      </c>
+      <c r="E2524" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="F2524" t="n">
+        <v>34</v>
+      </c>
+      <c r="G2524" t="n">
+        <v>48</v>
+      </c>
+      <c r="H2524" t="n">
+        <v>49</v>
+      </c>
+      <c r="I2524" t="n">
+        <v>59</v>
+      </c>
+      <c r="J2524" t="n">
+        <v>70</v>
+      </c>
+      <c r="K2524" t="n">
+        <v>12</v>
+      </c>
+      <c r="L2524" t="inlineStr"/>
+    </row>
+    <row r="2525">
+      <c r="A2525" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B2525" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C2525" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2525" t="n">
+        <v>31</v>
+      </c>
+      <c r="E2525" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="F2525" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2525" t="n">
+        <v>18</v>
+      </c>
+      <c r="H2525" t="n">
+        <v>26</v>
+      </c>
+      <c r="I2525" t="n">
+        <v>43</v>
+      </c>
+      <c r="J2525" t="n">
+        <v>51</v>
+      </c>
+      <c r="K2525" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2525" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>